<commit_message>
Add Novel/Flexpoint to June-26 M&A after deeper sweep (5 M&A total)
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-06-26.xlsx
+++ b/Weekly_Fintech_Deals_2026-06-26.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,15 +460,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
@@ -592,40 +592,46 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>Take-Private</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>22-Jun-26</t>
+          <t>23-Jun-26</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Entendre</t>
+          <t>Ramsdens Holdings</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>MoonPay</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+          <t>FirstCash Holdings</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>270</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>6.8</v>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>AI accounting agents automating bookkeeping and reporting for stablecoin and digital-asset businesses</t>
+          <t>UK pawnbroking, foreign-exchange, precious-metals and jewellery retailer (174 stores) -- specialty consumer finance</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -635,14 +641,14 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Terms undisclosed. Early-stage (last raised $4M seed 2023, in which MoonPay participated).</t>
+          <t>BORDERLINE FINTECH (high-street pawn/FX). 600p cash/sh (~609p incl. dividend); equity ~£206M (~$273M), EV ~£203M (~$270M). LTM (Mar-26) rev ~$200M, adj. EBITDA ~$40M -&gt; EV/EBITDA ~6.8x, EV/Rev ~1.35x. [computed]</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -652,22 +658,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Asset/Book Acquisition</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>24-Jun-26</t>
+          <t>22-Jun-26</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Policygenius (P&amp;C book)</t>
+          <t>Entendre</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Matic</t>
+          <t>MoonPay</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
@@ -675,7 +681,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>~30,000-policy property &amp; casualty insurance portfolio acquired by embedded insurtech Matic</t>
+          <t>AI accounting agents automating bookkeeping and reporting for stablecoin and digital-asset businesses</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -685,53 +691,47 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Book purchase price undisclosed; Matic also took an undisclosed minority growth investment from Primus Capital.</t>
+          <t>Terms undisclosed. Early-stage (last raised $4M seed 2023, in which MoonPay participated).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>InsurTech</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Take-Private</t>
+          <t>Asset/Book Acquisition</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>23-Jun-26</t>
+          <t>24-Jun-26</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ramsdens Holdings</t>
+          <t>Policygenius (P&amp;C book)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>FirstCash Holdings</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>270</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>6.8</v>
-      </c>
+          <t>Matic</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>UK pawnbroking, foreign-exchange, precious-metals and jewellery retailer (174 stores) -- specialty consumer finance</t>
+          <t>~30,000-policy property &amp; casualty insurance portfolio acquired by embedded insurtech Matic</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -741,17 +741,68 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE FINTECH (high-street pawn/FX). 600p cash/sh (~609p incl. dividend); equity ~£206M (~$273M), EV ~£203M (~$270M, ~small net debt). LTM (Mar-26) rev ~$200M, adj. EBITDA ~$40M -&gt; EV/EBITDA ~6.8x, EV/Rev ~1.35x. [computed]</t>
+          <t>Book purchase price undisclosed; Matic also took an undisclosed minority growth investment from Primus Capital.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>PE Strategic Investment</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>22-Jun-26</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Novel Financial Holdings</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Flexpoint Ford</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Diversified underwriting and insurance-services holding company managing reciprocal exchanges and stock insurers</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Minority/strategic PE investment, terms undisclosed (Flexpoint Asset Opportunity Fund III &amp; Insurance Opportunity Fund I). ~$2B annual gross written premium. Borderline (insurance holdco, not pure tech).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Balanced fintech+traditional descriptions for Ramsdens, Novel, Warp
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-06-26.xlsx
+++ b/Weekly_Fintech_Deals_2026-06-26.xlsx
@@ -472,7 +472,7 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="54" customWidth="1" min="12" max="12"/>
   </cols>
@@ -631,7 +631,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>UK pawnbroking, foreign-exchange, precious-metals and jewellery retailer (174 stores) -- specialty consumer finance</t>
+          <t>Consumer financial-services and currency-exchange specialist (foreign exchange, international money transfer, secured lending) built on a traditional pawnbroking, precious-metals and jewellery-retail business across 174 UK stores</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -781,7 +781,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Diversified underwriting and insurance-services holding company managing reciprocal exchanges and stock insurers</t>
+          <t>Technology-enabled underwriting and insurance-services platform managing reciprocal exchanges and traditional stock insurers (~$2B gross written premium)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -826,7 +826,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="54" customWidth="1" min="12" max="12"/>
   </cols>
@@ -1123,7 +1123,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>AI-native HR and payroll platform automating tax, compliance, and benefits for high-growth companies</t>
+          <t>AI-native payroll-payments, tax, and benefits-finance platform within a broader HR / human-capital-management suite for high-growth companies</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add MSCI/First Street and FusionIQ/Marstone to June-26 M&A (7 M&A total)
</commit_message>
<xml_diff>
--- a/Weekly_Fintech_Deals_2026-06-26.xlsx
+++ b/Weekly_Fintech_Deals_2026-06-26.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Growth Capital Raises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M&amp;A'!$A$1:$L$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Growth Capital Raises'!$A$1:$L$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
@@ -542,7 +542,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Banking &amp; Lending Tech</t>
+          <t>Asset &amp; Wealth Tech</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -557,17 +557,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>23-Jun-26</t>
+          <t>22-Jun-26</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Kasisto</t>
+          <t>Marstone</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Backbase</t>
+          <t>FusionIQ</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -575,7 +575,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Pioneer of agentic/conversational AI for banking, partnered with ~55 financial institutions across 16 countries</t>
+          <t>Digital wealth-management platform (digital advice, financial planning and wellness) for banks, credit unions, and wealth managers</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Terms undisclosed. Kasisto raised ~$92M to date (clients incl. JPMorgan, Standard Chartered, TD). No revenue disclosed.</t>
+          <t>Terms undisclosed (completed acquisition). Combines with FusionIQ's cloud-based wealth-management platform.</t>
         </is>
       </c>
     </row>
@@ -597,12 +597,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Take-Private</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -612,26 +612,20 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ramsdens Holdings</t>
+          <t>Kasisto</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>FirstCash Holdings</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>270</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>6.8</v>
-      </c>
+          <t>Backbase</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Consumer financial-services and currency-exchange specialist (foreign exchange, international money transfer, secured lending) built on a traditional pawnbroking, precious-metals and jewellery-retail business across 174 UK stores</t>
+          <t>Pioneer of agentic/conversational AI for banking, partnered with ~55 financial institutions across 16 countries</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -641,47 +635,53 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>BORDERLINE FINTECH (high-street pawn/FX). 600p cash/sh (~609p incl. dividend); equity ~£206M (~$273M), EV ~£203M (~$270M). LTM (Mar-26) rev ~$200M, adj. EBITDA ~$40M -&gt; EV/EBITDA ~6.8x, EV/Rev ~1.35x. [computed]</t>
+          <t>Terms undisclosed. Kasisto raised ~$92M to date (clients incl. JPMorgan, Standard Chartered, TD). No revenue disclosed.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Capital Markets Tech</t>
+          <t>Banking &amp; Lending Tech</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Strategic M&amp;A</t>
+          <t>Take-Private</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>22-Jun-26</t>
+          <t>23-Jun-26</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Entendre</t>
+          <t>Ramsdens Holdings</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>MoonPay</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+          <t>FirstCash Holdings</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>270</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>6.8</v>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>AI accounting agents automating bookkeeping and reporting for stablecoin and digital-asset businesses</t>
+          <t>Consumer financial-services and currency-exchange specialist (foreign exchange, international money transfer, secured lending) built on a traditional pawnbroking, precious-metals and jewellery-retail business across 174 UK stores</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -691,14 +691,14 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Terms undisclosed. Early-stage (last raised $4M seed 2023, in which MoonPay participated).</t>
+          <t>BORDERLINE FINTECH (high-street pawn/FX). 600p cash/sh (~609p incl. dividend); equity ~£206M (~$273M), EV ~£203M (~$270M). LTM (Mar-26) rev ~$200M, adj. EBITDA ~$40M -&gt; EV/EBITDA ~6.8x, EV/Rev ~1.35x. [computed]</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Capital Markets Tech</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Asset/Book Acquisition</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>24-Jun-26</t>
+          <t>22-Jun-26</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Policygenius (P&amp;C book)</t>
+          <t>Entendre</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Matic</t>
+          <t>MoonPay</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
@@ -731,7 +731,7 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>~30,000-policy property &amp; casualty insurance portfolio acquired by embedded insurtech Matic</t>
+          <t>AI accounting agents automating bookkeeping and reporting for stablecoin and digital-asset businesses</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -741,14 +741,14 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Book purchase price undisclosed; Matic also took an undisclosed minority growth investment from Primus Capital.</t>
+          <t>Terms undisclosed. Early-stage (last raised $4M seed 2023, in which MoonPay participated).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>InsurTech</t>
+          <t>Financial Info &amp; Analytics</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -758,51 +758,155 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PE Strategic Investment</t>
+          <t>Strategic M&amp;A</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>22-Jun-26</t>
+          <t>24-Jun-26</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Novel Financial Holdings</t>
+          <t>First Street</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Flexpoint Ford</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>MSCI</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>120</v>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
+          <t>Physics-based physical climate-risk data and analytics whose AI-enabled, multi-hazard models translate climate hazards into financial risk across 2B+ structures</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>$120M cash at closing + contingent earnouts (revenue-threshold-based, first 2 yrs). Target revenue/EBITDA not disclosed; reports in MSCI's Sustainability &amp; Climate segment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Asset/Book Acquisition</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>24-Jun-26</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Policygenius (P&amp;C book)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Matic</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>~30,000-policy property &amp; casualty insurance portfolio acquired by embedded insurtech Matic</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Book purchase price undisclosed; Matic also took an undisclosed minority growth investment from Primus Capital.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>InsurTech</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>PE Strategic Investment</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>22-Jun-26</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Novel Financial Holdings</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Flexpoint Ford</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>Technology-enabled underwriting and insurance-services platform managing reciprocal exchanges and traditional stock insurers (~$2B gross written premium)</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Minority/strategic PE investment, terms undisclosed (Flexpoint Asset Opportunity Fund III &amp; Insurance Opportunity Fund I). ~$2B annual gross written premium. Borderline (insurance holdco, not pure tech).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>